<commit_message>
1. CmdHelper added 2. PdfHelper v2 (with ai and ocr)
</commit_message>
<xml_diff>
--- a/FWUsefulPageObjects/TestCases/PDF/PDF Text Assert/Main.rvl.xlsx
+++ b/FWUsefulPageObjects/TestCases/PDF/PDF Text Assert/Main.rvl.xlsx
@@ -1,6 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fileVersion appName="libxl" rupBuild="5010000"/>
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -13,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="149" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="401" uniqueCount="73">
   <si>
     <t>Flow</t>
   </si>
@@ -148,6 +149,90 @@
   </si>
   <si>
     <t>PDF</t>
+  </si>
+  <si>
+    <t>SetPerferredMethod</t>
+  </si>
+  <si>
+    <t>method</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>ocr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check </t>
+  </si>
+  <si>
+    <t>Check 351</t>
+  </si>
+  <si>
+    <t>Img.pdf</t>
+  </si>
+  <si>
+    <t>351</t>
+  </si>
+  <si>
+    <t>ai</t>
+  </si>
+  <si>
+    <t>Check ELECTRON_ENABLE_LOGGING</t>
+  </si>
+  <si>
+    <t>ELECTRON_ENABLE_LOGGING</t>
+  </si>
+  <si>
+    <t>Img2.pdf</t>
+  </si>
+  <si>
+    <t>Check ELECTRON_ENABLE_LOGGING via OCR</t>
+  </si>
+  <si>
+    <t>Check ELECTRON_ENABLE_LOGGING via AI</t>
+  </si>
+  <si>
+    <t>Ocr</t>
+  </si>
+  <si>
+    <t>DoSetOcrOption</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>language</t>
+  </si>
+  <si>
+    <t>fr-FR</t>
+  </si>
+  <si>
+    <t>en-US</t>
+  </si>
+  <si>
+    <t>regex:ELECTRON.ENABLE.LOGGING</t>
+  </si>
+  <si>
+    <t>global.pdfLastError = "pdftoimage.js page count: "+pageNo;</t>
+  </si>
+  <si>
+    <t>regex:.*ELECTRON.ENABLE.LOGGING.*</t>
+  </si>
+  <si>
+    <t>UNStates.pdf</t>
+  </si>
+  <si>
+    <t>UNStatesImg.pdf</t>
+  </si>
+  <si>
+    <t>Find Solomon Islands</t>
+  </si>
+  <si>
+    <t>Solomon Islands</t>
   </si>
 </sst>
 </file>
@@ -168,7 +253,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="172">
+  <borders count="193">
     <border>
       <left/>
       <right/>
@@ -347,11 +432,32 @@
     <border/>
     <border/>
     <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="172">
+  <cellXfs count="193">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
@@ -524,6 +630,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="169" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="170" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="171" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="172" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="173" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="174" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="175" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="176" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="177" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="178" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="179" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="180" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="181" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="182" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="183" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="184" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="185" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="186" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="187" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="188" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="189" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="190" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="191" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="192" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -533,7 +660,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.34375" customWidth="true"/>
@@ -839,54 +966,579 @@
     </row>
     <row r="20">
       <c r="A20" s="121"/>
-      <c r="B20" s="122"/>
-      <c r="C20" s="123"/>
-      <c r="D20" s="124"/>
-      <c r="E20" s="125"/>
-      <c r="F20" s="126"/>
-      <c r="G20" s="127"/>
+      <c r="B20" s="122" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="123" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="124" t="s">
+        <v>60</v>
+      </c>
+      <c r="E20" s="125" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20" s="126" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="127" t="s">
+        <v>63</v>
+      </c>
       <c r="H20" s="128"/>
     </row>
     <row r="21">
-      <c r="A21" s="129"/>
-      <c r="B21" s="130"/>
-      <c r="C21" s="131"/>
-      <c r="D21" s="132"/>
-      <c r="E21" s="133"/>
-      <c r="F21" s="134"/>
-      <c r="G21" s="135"/>
-      <c r="H21" s="136"/>
+      <c r="A21" s="183"/>
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21" t="s">
+        <v>62</v>
+      </c>
+      <c r="F21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="137"/>
-      <c r="B22" s="138"/>
-      <c r="C22" s="139"/>
-      <c r="D22" s="140"/>
-      <c r="E22" s="141"/>
-      <c r="F22" s="142"/>
-      <c r="G22" s="143"/>
+      <c r="B22" s="138" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="139" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="140" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="141" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" s="142" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="143" t="s">
+        <v>48</v>
+      </c>
       <c r="H22" s="144"/>
     </row>
     <row r="23">
       <c r="A23" s="145"/>
-      <c r="B23" s="146"/>
-      <c r="C23" s="147"/>
-      <c r="D23" s="148"/>
-      <c r="E23" s="149"/>
-      <c r="F23" s="150"/>
-      <c r="G23" s="151"/>
+      <c r="B23" s="146" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="147" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="148" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="149" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23" s="150" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="151" t="s">
+        <v>50</v>
+      </c>
       <c r="H23" s="152"/>
     </row>
     <row r="24">
-      <c r="A24" s="153"/>
-      <c r="B24" s="154"/>
-      <c r="C24" s="155"/>
-      <c r="D24" s="156"/>
-      <c r="E24" s="157"/>
-      <c r="F24" s="158"/>
-      <c r="G24" s="159"/>
-      <c r="H24" s="160"/>
+      <c r="A24" s="173"/>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="174"/>
+      <c r="B25" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="182"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="181"/>
+      <c r="B27" t="s">
+        <v>3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" t="s">
+        <v>46</v>
+      </c>
+      <c r="F27" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="181"/>
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" t="s">
+        <v>30</v>
+      </c>
+      <c r="F28" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="181"/>
+      <c r="B29" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="181"/>
+      <c r="B30" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" t="s">
+        <v>22</v>
+      </c>
+      <c r="F30" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="153"/>
+      <c r="B31" s="154"/>
+      <c r="C31" s="155"/>
+      <c r="D31" s="156"/>
+      <c r="E31" s="157"/>
+      <c r="F31" s="158"/>
+      <c r="G31" s="159"/>
+      <c r="H31" s="160"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="180"/>
+      <c r="B32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="179"/>
+      <c r="B33" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" t="s">
+        <v>41</v>
+      </c>
+      <c r="E33" t="s">
+        <v>30</v>
+      </c>
+      <c r="F33" t="s">
+        <v>13</v>
+      </c>
+      <c r="G33" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="179"/>
+      <c r="B34" t="s">
+        <v>21</v>
+      </c>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="179"/>
+      <c r="B35" t="s">
+        <v>21</v>
+      </c>
+      <c r="E35" t="s">
+        <v>22</v>
+      </c>
+      <c r="F35" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="177"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="178"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="175"/>
+      <c r="B38" t="s">
+        <v>3</v>
+      </c>
+      <c r="C38" t="s">
+        <v>44</v>
+      </c>
+      <c r="D38" t="s">
+        <v>45</v>
+      </c>
+      <c r="E38" t="s">
+        <v>46</v>
+      </c>
+      <c r="F38" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="175"/>
+      <c r="B39" t="s">
+        <v>3</v>
+      </c>
+      <c r="C39" t="s">
+        <v>44</v>
+      </c>
+      <c r="D39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E39" t="s">
+        <v>30</v>
+      </c>
+      <c r="F39" t="s">
+        <v>13</v>
+      </c>
+      <c r="G39" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="175"/>
+      <c r="B40" t="s">
+        <v>21</v>
+      </c>
+      <c r="E40" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G40" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="175"/>
+      <c r="B41" t="s">
+        <v>21</v>
+      </c>
+      <c r="E41" t="s">
+        <v>22</v>
+      </c>
+      <c r="F41" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="176"/>
+      <c r="B44" t="s">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" t="s">
+        <v>45</v>
+      </c>
+      <c r="E44" t="s">
+        <v>46</v>
+      </c>
+      <c r="F44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G44" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="186"/>
+      <c r="B45" t="s">
+        <v>3</v>
+      </c>
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+      <c r="D45" t="s">
+        <v>39</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" t="s">
+        <v>43</v>
+      </c>
+      <c r="G45" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="186"/>
+      <c r="B46" t="s">
+        <v>3</v>
+      </c>
+      <c r="C46" t="s">
+        <v>15</v>
+      </c>
+      <c r="D46" t="s">
+        <v>16</v>
+      </c>
+      <c r="E46" t="s">
+        <v>17</v>
+      </c>
+      <c r="F46" t="s">
+        <v>18</v>
+      </c>
+      <c r="G46" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="186"/>
+      <c r="B47" t="s">
+        <v>21</v>
+      </c>
+      <c r="E47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F47" t="s">
+        <v>18</v>
+      </c>
+      <c r="G47" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="184"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="188"/>
+      <c r="B49" t="s">
+        <v>3</v>
+      </c>
+      <c r="C49" t="s">
+        <v>44</v>
+      </c>
+      <c r="D49" t="s">
+        <v>45</v>
+      </c>
+      <c r="E49" t="s">
+        <v>46</v>
+      </c>
+      <c r="F49" t="s">
+        <v>13</v>
+      </c>
+      <c r="G49" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="188"/>
+      <c r="B50" t="s">
+        <v>3</v>
+      </c>
+      <c r="C50" t="s">
+        <v>44</v>
+      </c>
+      <c r="D50" t="s">
+        <v>41</v>
+      </c>
+      <c r="E50" t="s">
+        <v>30</v>
+      </c>
+      <c r="F50" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="188"/>
+      <c r="B51" t="s">
+        <v>21</v>
+      </c>
+      <c r="E51" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="188"/>
+      <c r="B52" t="s">
+        <v>21</v>
+      </c>
+      <c r="E52" t="s">
+        <v>22</v>
+      </c>
+      <c r="F52" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="188"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="190"/>
+      <c r="B54" t="s">
+        <v>3</v>
+      </c>
+      <c r="C54" t="s">
+        <v>44</v>
+      </c>
+      <c r="D54" t="s">
+        <v>45</v>
+      </c>
+      <c r="E54" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="190"/>
+      <c r="B55" t="s">
+        <v>3</v>
+      </c>
+      <c r="C55" t="s">
+        <v>44</v>
+      </c>
+      <c r="D55" t="s">
+        <v>41</v>
+      </c>
+      <c r="E55" t="s">
+        <v>30</v>
+      </c>
+      <c r="F55" t="s">
+        <v>13</v>
+      </c>
+      <c r="G55" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="190"/>
+      <c r="B56" t="s">
+        <v>21</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>13</v>
+      </c>
+      <c r="G56" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="190"/>
+      <c r="B57" t="s">
+        <v>21</v>
+      </c>
+      <c r="E57" t="s">
+        <v>22</v>
+      </c>
+      <c r="F57" t="s">
+        <v>13</v>
+      </c>
+      <c r="G57" t="s">
+        <v>72</v>
+      </c>
     </row>
   </sheetData>
+  <tableParts/>
 </worksheet>
 </file>
</xml_diff>